<commit_message>
chore: update sample excel generator and templates to new 12-column format
</commit_message>
<xml_diff>
--- a/public/templates/mau-ho-so-me.xlsx
+++ b/public/templates/mau-ho-so-me.xlsx
@@ -398,162 +398,177 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:L4"/>
   <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="45.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" customWidth="1"/>
-    <col min="6" max="6" width="15.83203125" customWidth="1"/>
-    <col min="7" max="7" width="10.83203125" customWidth="1"/>
-    <col min="8" max="8" width="15.83203125" customWidth="1"/>
-    <col min="9" max="9" width="25.83203125" customWidth="1"/>
-    <col min="10" max="10" width="60.83203125" customWidth="1"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="25.83203125" customWidth="1"/>
+    <col min="4" max="4" width="25.83203125" customWidth="1"/>
+    <col min="5" max="5" width="60.83203125" customWidth="1"/>
+    <col min="6" max="6" width="25.83203125" customWidth="1"/>
+    <col min="7" max="7" width="25.83203125" customWidth="1"/>
+    <col min="8" max="8" width="10.83203125" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" customWidth="1"/>
+    <col min="10" max="10" width="10.83203125" customWidth="1"/>
+    <col min="11" max="11" width="15.83203125" customWidth="1"/>
+    <col min="12" max="12" width="30.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>Hộp số</v>
+      </c>
+      <c r="B1" t="str">
         <v>Hồ sơ số</v>
       </c>
-      <c r="B1" t="str">
+      <c r="C1" t="str">
+        <v>Số bản án/ quyết định</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Ngày bản án/ quyết định</v>
+      </c>
+      <c r="E1" t="str">
         <v>Tiêu đề</v>
       </c>
-      <c r="C1" t="str">
+      <c r="F1" t="str">
+        <v>Nguyên đơn/ người bị hại</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Bị cáo/ bị đơn</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Số tờ</v>
+      </c>
+      <c r="I1" t="str">
         <v>Loại án</v>
       </c>
-      <c r="D1" t="str">
+      <c r="J1" t="str">
         <v>Thời gian</v>
       </c>
-      <c r="E1" t="str">
-        <v>Số tờ</v>
-      </c>
-      <c r="F1" t="str">
+      <c r="K1" t="str">
         <v>THBQ</v>
       </c>
-      <c r="G1" t="str">
-        <v>Hộp số</v>
-      </c>
-      <c r="H1" t="str">
-        <v>MLHS</v>
-      </c>
-      <c r="I1" t="str">
+      <c r="L1" t="str">
         <v>Ghi chú</v>
       </c>
-      <c r="J1" t="str">
-        <v>:</v>
-      </c>
-    </row>
-    <row r="2" xml:space="preserve">
+    </row>
+    <row r="2">
       <c r="A2" t="str">
+        <v>H01</v>
+      </c>
+      <c r="B2" t="str">
         <v>2024/HS-ST/01</v>
       </c>
-      <c r="B2" t="str">
+      <c r="C2" t="str">
+        <v>45/2024/QĐ-ST</v>
+      </c>
+      <c r="D2" t="str">
+        <v>15/04/2024</v>
+      </c>
+      <c r="E2" t="str">
         <v>Vụ án Nguyễn Văn A và đồng phạm về tội Trộm cắp tài sản</v>
       </c>
-      <c r="C2" t="str">
+      <c r="F2" t="str">
+        <v>Công ty TNHH X</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Nguyễn Văn A, Trần Văn B</v>
+      </c>
+      <c r="H2">
+        <v>150</v>
+      </c>
+      <c r="I2" t="str">
         <v>Hình sự</v>
       </c>
-      <c r="D2">
+      <c r="J2">
         <v>2024</v>
       </c>
-      <c r="E2">
-        <v>150</v>
-      </c>
-      <c r="F2" t="str">
+      <c r="K2" t="str">
         <v>Vĩnh viễn</v>
       </c>
-      <c r="G2" t="str">
+      <c r="L2" t="str">
+        <v>Hồ sơ án điểm năm 2024</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
         <v>H01</v>
       </c>
-      <c r="H2" t="str">
-        <v>ML-2024-01</v>
-      </c>
-      <c r="I2" t="str">
-        <v>Hồ sơ án điểm năm 2024</v>
-      </c>
-      <c r="J2" t="str" xml:space="preserve">
-        <v xml:space="preserve">Về việc: Vụ án Nguyễn Văn A và đồng phạm về tội Trộm cắp tài sản
-Bị cáo: Nguyễn Văn A, Trần Văn B
-QDTHS: 45/2024/QĐ-ST
-Ngày: 15/04/2024</v>
-      </c>
-    </row>
-    <row r="3" xml:space="preserve">
-      <c r="A3" t="str">
+      <c r="B3" t="str">
         <v>2024/DS-ST/02</v>
       </c>
-      <c r="B3" t="str">
+      <c r="C3" t="str">
+        <v>12/2024/DS-ST</v>
+      </c>
+      <c r="D3" t="str">
+        <v>20/05/2024</v>
+      </c>
+      <c r="E3" t="str">
         <v>Vụ án tranh chấp hợp đồng chuyển nhượng quyền sử dụng đất</v>
       </c>
-      <c r="C3" t="str">
+      <c r="F3" t="str">
+        <v>Lê Thị C</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Phạm Văn D</v>
+      </c>
+      <c r="H3">
+        <v>85</v>
+      </c>
+      <c r="I3" t="str">
         <v>Dân sự</v>
       </c>
-      <c r="D3">
+      <c r="J3">
         <v>2024</v>
       </c>
-      <c r="E3">
-        <v>85</v>
-      </c>
-      <c r="F3" t="str">
+      <c r="K3" t="str">
         <v>50 năm</v>
       </c>
-      <c r="G3" t="str">
-        <v>H01</v>
-      </c>
-      <c r="H3" t="str">
-        <v>ML-2024-01</v>
-      </c>
-      <c r="I3" t="str">
+      <c r="L3" t="str">
         <v>Đã thi hành án xong</v>
       </c>
-      <c r="J3" t="str" xml:space="preserve">
-        <v xml:space="preserve">Về việc: Vụ án tranh chấp hợp đồng chuyển nhượng quyền sử dụng đất
-Nguyên đơn: Lê Thị C
-Bị đơn: Phạm Văn D
-Số: 12/2024/DS-ST
-Ngày: 20/05/2024</v>
-      </c>
-    </row>
-    <row r="4" xml:space="preserve">
+    </row>
+    <row r="4">
       <c r="A4" t="str">
+        <v>H02</v>
+      </c>
+      <c r="B4" t="str">
         <v>2024/HC-ST/03</v>
       </c>
-      <c r="B4" t="str">
+      <c r="C4" t="str">
+        <v>08/2024/HC-ST</v>
+      </c>
+      <c r="D4" t="str">
+        <v>10/06/2024</v>
+      </c>
+      <c r="E4" t="str">
         <v>Vụ án khiếu kiện quyết định xử phạt hành chính trong lĩnh vực đất đai</v>
       </c>
-      <c r="C4" t="str">
+      <c r="F4" t="str">
+        <v>Hoàng Văn E</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Ủy ban nhân dân quận X</v>
+      </c>
+      <c r="H4">
+        <v>60</v>
+      </c>
+      <c r="I4" t="str">
         <v>Hành chính</v>
       </c>
-      <c r="D4">
+      <c r="J4">
         <v>2024</v>
       </c>
-      <c r="E4">
-        <v>60</v>
-      </c>
-      <c r="F4" t="str">
+      <c r="K4" t="str">
         <v>15 năm</v>
       </c>
-      <c r="G4" t="str">
-        <v>H02</v>
-      </c>
-      <c r="H4" t="str">
-        <v>ML-2024-02</v>
-      </c>
-      <c r="I4" t="str">
+      <c r="L4" t="str">
         <v>Lưu trữ tại kho B</v>
-      </c>
-      <c r="J4" t="str" xml:space="preserve">
-        <v xml:space="preserve">Về việc: Vụ án khiếu kiện quyết định xử phạt hành chính trong lĩnh vực đất đai
-Nguyên đơn: Hoàng Văn E
-Bị đơn: Ủy ban nhân dân quận X
-Số: 08/2024/HC-ST
-Ngày: 10/06/2024</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L4"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore: update public template with 5 case types sample data
</commit_message>
<xml_diff>
--- a/public/templates/mau-ho-so-me.xlsx
+++ b/public/templates/mau-ho-so-me.xlsx
@@ -398,18 +398,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L6"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="25.83203125" customWidth="1"/>
-    <col min="4" max="4" width="25.83203125" customWidth="1"/>
-    <col min="5" max="5" width="60.83203125" customWidth="1"/>
-    <col min="6" max="6" width="25.83203125" customWidth="1"/>
-    <col min="7" max="7" width="25.83203125" customWidth="1"/>
+    <col min="3" max="3" width="24.83203125" customWidth="1"/>
+    <col min="4" max="4" width="24.83203125" customWidth="1"/>
+    <col min="5" max="5" width="45.83203125" customWidth="1"/>
+    <col min="6" max="6" width="30.83203125" customWidth="1"/>
+    <col min="7" max="7" width="30.83203125" customWidth="1"/>
     <col min="8" max="8" width="10.83203125" customWidth="1"/>
-    <col min="9" max="9" width="12.83203125" customWidth="1"/>
-    <col min="10" max="10" width="10.83203125" customWidth="1"/>
+    <col min="9" max="9" width="22.83203125" customWidth="1"/>
+    <col min="10" max="10" width="12.83203125" customWidth="1"/>
     <col min="11" max="11" width="15.83203125" customWidth="1"/>
     <col min="12" max="12" width="30.83203125" customWidth="1"/>
   </cols>
@@ -460,7 +460,7 @@
         <v>2024/HS-ST/01</v>
       </c>
       <c r="C2" t="str">
-        <v>45/2024/QĐ-ST</v>
+        <v>45/2024/HS-ST</v>
       </c>
       <c r="D2" t="str">
         <v>15/04/2024</v>
@@ -469,13 +469,13 @@
         <v>Vụ án Nguyễn Văn A và đồng phạm về tội Trộm cắp tài sản</v>
       </c>
       <c r="F2" t="str">
-        <v>Công ty TNHH X</v>
+        <v>Công ty TNHH Xây dựng Việt Nhật</v>
       </c>
       <c r="G2" t="str">
         <v>Nguyễn Văn A, Trần Văn B</v>
       </c>
       <c r="H2">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="I2" t="str">
         <v>Hình sự</v>
@@ -510,10 +510,10 @@
         <v>Lê Thị C</v>
       </c>
       <c r="G3" t="str">
-        <v>Phạm Văn D</v>
+        <v>Phạm Văn D, Vũ Thị E</v>
       </c>
       <c r="H3">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="I3" t="str">
         <v>Dân sự</v>
@@ -542,7 +542,7 @@
         <v>10/06/2024</v>
       </c>
       <c r="E4" t="str">
-        <v>Vụ án khiếu kiện quyết định xử phạt hành chính trong lĩnh vực đất đai</v>
+        <v>Vụ án khiếu kiện quyết định xử phạt vi phạm hành chính trong lĩnh vực đất đai</v>
       </c>
       <c r="F4" t="str">
         <v>Hoàng Văn E</v>
@@ -551,7 +551,7 @@
         <v>Ủy ban nhân dân quận X</v>
       </c>
       <c r="H4">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="I4" t="str">
         <v>Hành chính</v>
@@ -566,25 +566,101 @@
         <v>Lưu trữ tại kho B</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>H02</v>
+      </c>
+      <c r="B5" t="str">
+        <v>2024/HNGĐ-ST/04</v>
+      </c>
+      <c r="C5" t="str">
+        <v>19/2024/HNGĐ-ST</v>
+      </c>
+      <c r="D5" t="str">
+        <v>25/07/2024</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Vụ án tranh chấp ly hôn, chia tài sản chung và quyền nuôi con</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Trần Thị Thu Trang</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Đỗ Văn Hùng</v>
+      </c>
+      <c r="H5">
+        <v>55</v>
+      </c>
+      <c r="I5" t="str">
+        <v>Hôn nhân gia đình</v>
+      </c>
+      <c r="J5">
+        <v>2024</v>
+      </c>
+      <c r="K5" t="str">
+        <v>20 năm</v>
+      </c>
+      <c r="L5" t="str">
+        <v>Đã hòa giải không thành</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>H03</v>
+      </c>
+      <c r="B6" t="str">
+        <v>2024/KDTM-ST/05</v>
+      </c>
+      <c r="C6" t="str">
+        <v>05/2024/KDTM-ST</v>
+      </c>
+      <c r="D6" t="str">
+        <v>12/08/2024</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Vụ án tranh chấp hợp đồng mua bán hàng hóa và bồi thường thiệt hại</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Công ty Cổ phần Thương mại Alpha</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Công ty TNHH Xuất Nhập khẩu Beta</v>
+      </c>
+      <c r="H6">
+        <v>110</v>
+      </c>
+      <c r="I6" t="str">
+        <v>Kinh doanh thương mại</v>
+      </c>
+      <c r="J6">
+        <v>2024</v>
+      </c>
+      <c r="K6" t="str">
+        <v>70 năm</v>
+      </c>
+      <c r="L6" t="str">
+        <v>Án kinh doanh thương mại sơ thẩm</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L6"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H8"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
     <col min="3" max="3" width="45.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" customWidth="1"/>
+    <col min="4" max="4" width="20.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
     <col min="6" max="6" width="10.83203125" customWidth="1"/>
-    <col min="7" max="7" width="18.83203125" customWidth="1"/>
-    <col min="8" max="8" width="20.83203125" customWidth="1"/>
+    <col min="7" max="7" width="20.83203125" customWidth="1"/>
+    <col min="8" max="8" width="25.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -630,7 +706,7 @@
         <v>2024</v>
       </c>
       <c r="F2">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G2" t="str">
         <v>Vĩnh viễn</v>
@@ -656,13 +732,13 @@
         <v>2024</v>
       </c>
       <c r="F3">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="G3" t="str">
         <v>Vĩnh viễn</v>
       </c>
       <c r="H3" t="str">
-        <v>Bản chính</v>
+        <v>Bản chính có đóng dấu</v>
       </c>
     </row>
     <row r="4">
@@ -682,7 +758,7 @@
         <v>2024</v>
       </c>
       <c r="F4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G4" t="str">
         <v>50 năm</v>
@@ -699,7 +775,7 @@
         <v>VB-02</v>
       </c>
       <c r="C5" t="str">
-        <v>Hợp đồng chuyển nhượng quyền sử dụng đất</v>
+        <v>Hợp đồng chuyển nhượng quyền sử dụng đất có công chứng</v>
       </c>
       <c r="D5" t="str">
         <v>Dân sự</v>
@@ -708,7 +784,7 @@
         <v>2024</v>
       </c>
       <c r="F5">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G5" t="str">
         <v>50 năm</v>
@@ -717,9 +793,87 @@
         <v>Bản sao công chứng</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>2024/HC-ST/03</v>
+      </c>
+      <c r="B6" t="str">
+        <v>VB-01</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Quyết định xử phạt vi phạm hành chính số 102/QĐ-XPHC</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Hành chính</v>
+      </c>
+      <c r="E6">
+        <v>2024</v>
+      </c>
+      <c r="F6">
+        <v>8</v>
+      </c>
+      <c r="G6" t="str">
+        <v>15 năm</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Bản sao y</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>2024/HNGĐ-ST/04</v>
+      </c>
+      <c r="B7" t="str">
+        <v>VB-01</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Biên bản hòa giải không thành tại Tòa án</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Hôn nhân gia đình</v>
+      </c>
+      <c r="E7">
+        <v>2024</v>
+      </c>
+      <c r="F7">
+        <v>5</v>
+      </c>
+      <c r="G7" t="str">
+        <v>20 năm</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Bản gốc</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>2024/KDTM-ST/05</v>
+      </c>
+      <c r="B8" t="str">
+        <v>VB-01</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Hợp đồng mua bán quốc tế số 88/2023/HDMB</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Kinh doanh thương mại</v>
+      </c>
+      <c r="E8">
+        <v>2024</v>
+      </c>
+      <c r="F8">
+        <v>15</v>
+      </c>
+      <c r="G8" t="str">
+        <v>70 năm</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Song ngữ Việt - Anh</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>